<commit_message>
Added effect sizes for a few plots
</commit_message>
<xml_diff>
--- a/SFN/oafemScatter.xlsx
+++ b/SFN/oafemScatter.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11010"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/avidachs/Documents/GitHub/rf1-sra-trust/SFN/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/coopersharp/Desktop/Smith Neuro Lab/GitHub/rf1-sra-trust/SFN/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAD4F8EB-3457-9648-9165-48F0D3C13B0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC7AB509-5421-3E4F-A590-BCB69E02C66D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="980" windowWidth="24180" windowHeight="15620" xr2:uid="{06A61F8C-AD50-8240-932B-24E52E3BA800}"/>
+    <workbookView xWindow="2300" yWindow="9120" windowWidth="40960" windowHeight="22540" activeTab="1" xr2:uid="{06A61F8C-AD50-8240-932B-24E52E3BA800}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -27,8 +28,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -36,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="6">
   <si>
     <t>age</t>
   </si>
@@ -49,13 +48,27 @@
   <si>
     <t>oafem</t>
   </si>
+  <si>
+    <t>R</t>
+  </si>
+  <si>
+    <t>std</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -71,7 +84,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -79,12 +92,37 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -398,11 +436,111 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53375E68-07BE-624E-B3DA-934CD129D8BC}">
-  <dimension ref="A1:D90"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F343160-525B-5042-A449-F38A05515319}">
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" s="3"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" s="1"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" s="1"/>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" s="1"/>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10" s="1"/>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11" s="1"/>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" s="1"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13" s="1"/>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14" s="1"/>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+    </row>
+    <row r="15" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53375E68-07BE-624E-B3DA-934CD129D8BC}">
+  <dimension ref="A1:I71"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -415,8 +553,17 @@
       <c r="D1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="G1" t="s">
+        <v>4</v>
+      </c>
+      <c r="H1" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>0</v>
       </c>
@@ -429,8 +576,16 @@
       <c r="D2">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="G2">
+        <f>CORREL(A2:A71, B2:B71)</f>
+        <v>-0.21559755675172182</v>
+      </c>
+      <c r="I2">
+        <f>CORREL(B2:B71, C2:C71)</f>
+        <v>-2.6461634288497855E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>0</v>
       </c>
@@ -444,7 +599,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>36</v>
       </c>
@@ -458,7 +613,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>2</v>
       </c>
@@ -472,7 +627,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>0</v>
       </c>
@@ -486,7 +641,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>0</v>
       </c>
@@ -500,7 +655,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>11</v>
       </c>
@@ -514,7 +669,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>19</v>
       </c>
@@ -528,7 +683,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>4</v>
       </c>
@@ -542,7 +697,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>9</v>
       </c>
@@ -556,7 +711,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>11</v>
       </c>
@@ -570,7 +725,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>15</v>
       </c>
@@ -584,7 +739,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>0</v>
       </c>
@@ -598,7 +753,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>8</v>
       </c>
@@ -612,7 +767,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>0</v>
       </c>
@@ -1388,158 +1543,6 @@
       </c>
       <c r="B71">
         <v>62.91</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A72" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="B72" t="e">
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A73" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="B73" t="e">
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A74" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="B74" t="e">
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A75" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="B75" t="e">
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A76" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="B76" t="e">
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A77" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="B77" t="e">
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A78" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="B78" t="e">
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A79" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="B79" t="e">
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A80" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="B80" t="e">
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A81" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="B81" t="e">
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A82" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="B82" t="e">
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A83" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="B83" t="e">
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A84" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="B84" t="e">
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A85" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="B85" t="e">
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A86" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="B86" t="e">
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A87" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="B87" t="e">
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A88" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="B88" t="e">
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A89" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="B89" t="e">
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A90" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="B90" t="e">
-        <v>#N/A</v>
       </c>
     </row>
   </sheetData>

</xml_diff>